<commit_message>
Remove unused Excel import components and routes - Clean up UAE and Amazon10 Excel imports - Remove UaeExcelImport and Amazon10ExcelImport components - Remove related routes from App.jsx and admin dashboard - Fix ApiDebug import error
</commit_message>
<xml_diff>
--- a/Products.xlsx
+++ b/Products.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abc\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Amazon Gymkhana-Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD1A793-953A-4904-BC8B-F51039B55863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4635" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK SHARK BRAND PRODUCT" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -6561,7 +6561,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -6903,7 +6903,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AD185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -23348,13 +23348,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>